<commit_message>
unpublished modules are locked
</commit_message>
<xml_diff>
--- a/I-READ-BackendAPI/students_bulk.xlsx
+++ b/I-READ-BackendAPI/students_bulk.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <r>
       <rPr>
@@ -121,70 +121,73 @@
     <t>Address</t>
   </si>
   <si>
+    <t>chanlumz</t>
+  </si>
+  <si>
+    <t>chnlum03@gmail.com</t>
+  </si>
+  <si>
+    <t>LouisPWiread</t>
+  </si>
+  <si>
     <t>chanlum</t>
   </si>
   <si>
-    <t>chnlum03@gmail.com</t>
-  </si>
-  <si>
-    <t>LouisPWiread</t>
-  </si>
-  <si>
-    <t>louis</t>
-  </si>
-  <si>
     <t>christian</t>
   </si>
   <si>
-    <t>lum</t>
+    <t>lums</t>
   </si>
   <si>
     <t>STEM</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>1433 taft ave ermita manila</t>
+  </si>
+  <si>
+    <t>gab_balma</t>
+  </si>
+  <si>
+    <t>gabalma@gmail.com</t>
+  </si>
+  <si>
+    <t>gbalma2003</t>
+  </si>
+  <si>
+    <t>gab</t>
+  </si>
+  <si>
+    <t>balma</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>cidivin</t>
+  </si>
+  <si>
+    <t>chloediv@gmail.com</t>
+  </si>
+  <si>
+    <t>Chloe54321</t>
+  </si>
+  <si>
+    <t>chloe</t>
+  </si>
+  <si>
+    <t>isobel</t>
+  </si>
+  <si>
+    <t>div</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
-    <t>1433 taft ave ermita manila</t>
-  </si>
-  <si>
-    <t>gab_balma</t>
-  </si>
-  <si>
-    <t>gabalma@gmail.com</t>
-  </si>
-  <si>
-    <t>gbalma2003</t>
-  </si>
-  <si>
-    <t>gab</t>
-  </si>
-  <si>
-    <t>balma</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>Quezon City</t>
-  </si>
-  <si>
-    <t>cidivin</t>
-  </si>
-  <si>
-    <t>chloediv@gmail.com</t>
-  </si>
-  <si>
-    <t>Chloe54321</t>
-  </si>
-  <si>
-    <t>chloe</t>
-  </si>
-  <si>
-    <t>isobel</t>
-  </si>
-  <si>
-    <t>div</t>
+    <t>Talon Singko</t>
   </si>
   <si>
     <t>ellaespique</t>
@@ -199,10 +202,100 @@
     <t>ella</t>
   </si>
   <si>
+    <t>mika</t>
+  </si>
+  <si>
     <t>espique</t>
   </si>
   <si>
     <t>ABM</t>
+  </si>
+  <si>
+    <t>molaguera</t>
+  </si>
+  <si>
+    <t>mark@gmail.com</t>
+  </si>
+  <si>
+    <t>markPW03</t>
+  </si>
+  <si>
+    <t>mark</t>
+  </si>
+  <si>
+    <t>olaguera</t>
+  </si>
+  <si>
+    <t>Pasig City</t>
+  </si>
+  <si>
+    <t>janesmith</t>
+  </si>
+  <si>
+    <t>janesmith@gmail.com</t>
+  </si>
+  <si>
+    <t>janePW01</t>
+  </si>
+  <si>
+    <t>jane</t>
+  </si>
+  <si>
+    <t>marie</t>
+  </si>
+  <si>
+    <t>smith</t>
+  </si>
+  <si>
+    <t>carlosr</t>
+  </si>
+  <si>
+    <t>carlosr@gmail.com</t>
+  </si>
+  <si>
+    <t>carlosPW02</t>
+  </si>
+  <si>
+    <t>carlos</t>
+  </si>
+  <si>
+    <t>reyes</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Manila</t>
+  </si>
+  <si>
+    <t>sharondiv</t>
+  </si>
+  <si>
+    <t>sharondiv@gmail.com</t>
+  </si>
+  <si>
+    <t>sharon12345</t>
+  </si>
+  <si>
+    <t>sharon</t>
+  </si>
+  <si>
+    <t>chuckgeorge</t>
+  </si>
+  <si>
+    <t>chuckgeorge@gmail.com</t>
+  </si>
+  <si>
+    <t>chuckIREADacc</t>
+  </si>
+  <si>
+    <t>chuck</t>
+  </si>
+  <si>
+    <t>george</t>
+  </si>
+  <si>
+    <t>Ermita Manila</t>
   </si>
 </sst>
 </file>
@@ -298,6 +391,20 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -311,20 +418,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -345,12 +438,12 @@
     <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="bottom"/>
     </xf>
@@ -360,13 +453,13 @@
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="9" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="9" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="6" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="9" fillId="4" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="6" fillId="4" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -594,7 +687,7 @@
     <col customWidth="1" min="2" max="2" width="22.38"/>
     <col customWidth="1" min="3" max="3" width="14.5"/>
     <col customWidth="1" min="7" max="7" width="13.63"/>
-    <col customWidth="1" min="8" max="8" width="23.13"/>
+    <col customWidth="1" min="8" max="8" width="22.13"/>
     <col customWidth="1" min="9" max="9" width="24.38"/>
     <col customWidth="1" min="10" max="10" width="21.75"/>
   </cols>
@@ -699,7 +792,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="17" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="17" t="s">
@@ -714,13 +807,13 @@
       <c r="E12" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="17" t="s">
         <v>17</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="H12" s="17" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="11">
@@ -753,81 +846,211 @@
         <v>26</v>
       </c>
       <c r="I13" s="19">
-        <v>38292.0</v>
-      </c>
-      <c r="J13" s="18" t="s">
-        <v>27</v>
+        <v>38147.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="D14" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="E14" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="F14" s="18" t="s">
         <v>32</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>33</v>
       </c>
       <c r="G14" s="18" t="s">
         <v>18</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="I14" s="19">
         <v>37926.0</v>
       </c>
+      <c r="J14" s="18" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>39</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="I15" s="19">
-        <v>37897.0</v>
+        <v>38000.0</v>
       </c>
     </row>
     <row r="16">
-      <c r="I16" s="1"/>
+      <c r="A16" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="I16" s="19">
+        <v>37915.0</v>
+      </c>
+      <c r="J16" s="18" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="17">
-      <c r="I17" s="1"/>
+      <c r="A17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I17" s="19">
+        <v>38042.0</v>
+      </c>
     </row>
     <row r="18">
-      <c r="I18" s="1"/>
+      <c r="A18" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="I18" s="19">
+        <v>38126.0</v>
+      </c>
+      <c r="J18" s="18" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="19">
-      <c r="I19" s="1"/>
+      <c r="A19" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I19" s="19">
+        <v>38147.0</v>
+      </c>
     </row>
     <row r="20">
-      <c r="I20" s="1"/>
+      <c r="A20" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I20" s="19">
+        <v>37844.0</v>
+      </c>
+      <c r="J20" s="18" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="21">
       <c r="I21" s="1"/>

</xml_diff>